<commit_message>
chore: auto-generate derived docs and explorer data
</commit_message>
<xml_diff>
--- a/docs/src/reference/data-dictionaries/C_Dict.xlsx
+++ b/docs/src/reference/data-dictionaries/C_Dict.xlsx
@@ -10741,12 +10741,12 @@
       </c>
       <c r="Z138" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA138" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB138" t="inlineStr"/>
@@ -10805,12 +10805,12 @@
       </c>
       <c r="Z139" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA139" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB139" t="inlineStr"/>
@@ -10869,12 +10869,12 @@
       </c>
       <c r="Z140" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA140" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB140" t="inlineStr"/>
@@ -10933,12 +10933,12 @@
       </c>
       <c r="Z141" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA141" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB141" t="inlineStr"/>
@@ -10997,12 +10997,12 @@
       </c>
       <c r="Z142" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA142" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB142" t="inlineStr"/>
@@ -11061,12 +11061,12 @@
       </c>
       <c r="Z143" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA143" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB143" t="inlineStr"/>
@@ -11125,12 +11125,12 @@
       </c>
       <c r="Z144" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA144" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB144" t="inlineStr"/>
@@ -11189,12 +11189,12 @@
       </c>
       <c r="Z145" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA145" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB145" t="inlineStr"/>
@@ -11253,12 +11253,12 @@
       </c>
       <c r="Z146" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA146" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB146" t="inlineStr"/>
@@ -11317,12 +11317,12 @@
       </c>
       <c r="Z147" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA147" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB147" t="inlineStr"/>
@@ -11381,12 +11381,12 @@
       </c>
       <c r="Z148" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA148" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB148" t="inlineStr"/>
@@ -11445,12 +11445,12 @@
       </c>
       <c r="Z149" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA149" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB149" t="inlineStr"/>
@@ -11509,12 +11509,12 @@
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB150" t="inlineStr"/>
@@ -11573,12 +11573,12 @@
       </c>
       <c r="Z151" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA151" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB151" t="inlineStr"/>
@@ -11637,12 +11637,12 @@
       </c>
       <c r="Z152" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA152" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB152" t="inlineStr"/>
@@ -11701,12 +11701,12 @@
       </c>
       <c r="Z153" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA153" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB153" t="inlineStr"/>
@@ -11765,12 +11765,12 @@
       </c>
       <c r="Z154" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA154" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB154" t="inlineStr"/>
@@ -11829,12 +11829,12 @@
       </c>
       <c r="Z155" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA155" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB155" t="inlineStr"/>
@@ -11893,12 +11893,12 @@
       </c>
       <c r="Z156" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA156" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB156" t="inlineStr"/>
@@ -11957,12 +11957,12 @@
       </c>
       <c r="Z157" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA157" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB157" t="inlineStr"/>
@@ -12021,12 +12021,12 @@
       </c>
       <c r="Z158" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA158" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB158" t="inlineStr"/>
@@ -12085,12 +12085,12 @@
       </c>
       <c r="Z159" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA159" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB159" t="inlineStr"/>
@@ -12149,12 +12149,12 @@
       </c>
       <c r="Z160" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA160" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB160" t="inlineStr"/>
@@ -12213,12 +12213,12 @@
       </c>
       <c r="Z161" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA161" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB161" t="inlineStr"/>
@@ -12277,12 +12277,12 @@
       </c>
       <c r="Z162" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA162" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB162" t="inlineStr"/>
@@ -12341,12 +12341,12 @@
       </c>
       <c r="Z163" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA163" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB163" t="inlineStr"/>
@@ -12405,12 +12405,12 @@
       </c>
       <c r="Z164" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA164" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB164" t="inlineStr"/>
@@ -12469,12 +12469,12 @@
       </c>
       <c r="Z165" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA165" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB165" t="inlineStr"/>
@@ -12533,12 +12533,12 @@
       </c>
       <c r="Z166" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA166" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB166" t="inlineStr"/>
@@ -12597,12 +12597,12 @@
       </c>
       <c r="Z167" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA167" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB167" t="inlineStr"/>
@@ -12661,12 +12661,12 @@
       </c>
       <c r="Z168" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA168" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB168" t="inlineStr"/>
@@ -12725,12 +12725,12 @@
       </c>
       <c r="Z169" t="inlineStr">
         <is>
-          <t>SAMSHA 2019, 2021; Vivitrol 2020; OSRM 2020;</t>
+          <t>SAMSHA 2019, 2021, 2025; Vivitrol 2020; OSRM 2020, 2025;</t>
         </is>
       </c>
       <c r="AA169" t="inlineStr">
         <is>
-          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019; Vivitrol, 2020; Open Source Routing Machine, 2020</t>
+          <t>U.S. Substance Abuse and Mental Health Services Administration, Treatment Locator Tool, 2019, 2025; Vivitrol, 2020; Open Source Routing Machine, 2020, 2025;</t>
         </is>
       </c>
       <c r="AB169" t="inlineStr"/>

</xml_diff>